<commit_message>
Added sample-based sound effects when 16K of sideways RAM is detected. Changes include:  - Introduced Sample.6502 which encapsulates the sample playback functionality.  - Added WAVConverter project that converts three sound effect WAV files to a compressed pcm data file.  - Updated LevelEditor, adding an additional level setting. Also renamed coefficients to settings.
</commit_message>
<xml_diff>
--- a/Memory.xlsx
+++ b/Memory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Beeb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED29658-03D7-4DC2-995F-FAAF7109DB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E5EAC4E-741D-4B83-BA2D-D5DEE8403802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
+    <workbookView xWindow="12950" yWindow="3250" windowWidth="24870" windowHeight="17050" xr2:uid="{C0DF3A0D-E6A9-4F13-8EDD-5DE46AD6E0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="73">
   <si>
     <t>Quantity</t>
   </si>
@@ -286,12 +286,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="32">
@@ -780,51 +786,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -833,7 +799,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -843,30 +809,66 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1213,35 +1215,35 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="88" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="57" t="s">
+      <c r="C2" s="90" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="56" t="s">
+      <c r="E2" s="84" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="59"/>
-      <c r="G2" s="56" t="s">
+      <c r="F2" s="87"/>
+      <c r="G2" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="57"/>
-      <c r="I2" s="58" t="s">
+      <c r="H2" s="85"/>
+      <c r="I2" s="86" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="59"/>
-      <c r="K2" s="56" t="s">
+      <c r="J2" s="87"/>
+      <c r="K2" s="84" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="57"/>
-      <c r="M2" s="58" t="s">
+      <c r="L2" s="85"/>
+      <c r="M2" s="86" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="59"/>
+      <c r="N2" s="87"/>
       <c r="O2" s="43" t="s">
         <v>6</v>
       </c>
@@ -1252,35 +1254,35 @@
       <c r="R2" s="15"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B3" s="67"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="61" t="s">
+      <c r="B3" s="89"/>
+      <c r="C3" s="91"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="91" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="63"/>
-      <c r="G3" s="61" t="s">
+      <c r="F3" s="93"/>
+      <c r="G3" s="91" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="62"/>
+      <c r="H3" s="92"/>
       <c r="I3" s="41"/>
       <c r="J3" s="40"/>
-      <c r="K3" s="61" t="s">
+      <c r="K3" s="91" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="62"/>
-      <c r="M3" s="63" t="s">
+      <c r="L3" s="92"/>
+      <c r="M3" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="N3" s="63"/>
+      <c r="N3" s="93"/>
       <c r="O3" s="42"/>
       <c r="P3" s="24"/>
       <c r="R3" s="15"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B4" s="67"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="62"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="91"/>
+      <c r="D4" s="92"/>
       <c r="E4" s="21" t="s">
         <v>0</v>
       </c>
@@ -1381,10 +1383,10 @@
       <c r="D6" s="5">
         <v>48</v>
       </c>
-      <c r="E6" s="65">
-        <v>0</v>
-      </c>
-      <c r="F6" s="65">
+      <c r="E6" s="30">
+        <v>0</v>
+      </c>
+      <c r="F6" s="30">
         <f>E6*$D6</f>
         <v>0</v>
       </c>
@@ -1395,10 +1397,10 @@
         <f>G6*$D6</f>
         <v>0</v>
       </c>
-      <c r="I6" s="65">
+      <c r="I6" s="30">
         <v>1</v>
       </c>
-      <c r="J6" s="65">
+      <c r="J6" s="30">
         <f>I6*$D6</f>
         <v>48</v>
       </c>
@@ -1409,10 +1411,10 @@
         <f>K6*$D6</f>
         <v>0</v>
       </c>
-      <c r="M6" s="65">
-        <v>0</v>
-      </c>
-      <c r="N6" s="65">
+      <c r="M6" s="30">
+        <v>0</v>
+      </c>
+      <c r="N6" s="30">
         <f>M6*$D6</f>
         <v>0</v>
       </c>
@@ -1435,10 +1437,10 @@
         <f>(24*32/4)</f>
         <v>192</v>
       </c>
-      <c r="E7" s="65">
+      <c r="E7" s="30">
         <v>1</v>
       </c>
-      <c r="F7" s="65">
+      <c r="F7" s="30">
         <f t="shared" ref="F7" si="0">E7*$D7</f>
         <v>192</v>
       </c>
@@ -1449,10 +1451,10 @@
         <f t="shared" ref="H7" si="1">G7*$D7</f>
         <v>192</v>
       </c>
-      <c r="I7" s="65">
+      <c r="I7" s="30">
         <v>2</v>
       </c>
-      <c r="J7" s="65">
+      <c r="J7" s="30">
         <f t="shared" ref="J7" si="2">I7*$D7</f>
         <v>384</v>
       </c>
@@ -1463,10 +1465,10 @@
         <f t="shared" ref="L7" si="3">K7*$D7</f>
         <v>960</v>
       </c>
-      <c r="M7" s="65">
+      <c r="M7" s="30">
         <v>2</v>
       </c>
-      <c r="N7" s="65">
+      <c r="N7" s="30">
         <f t="shared" ref="N7" si="4">M7*$D7</f>
         <v>384</v>
       </c>
@@ -1884,7 +1886,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="12"/>
-      <c r="J16" s="64">
+      <c r="J16" s="16">
         <f>J15-J14</f>
         <v>0</v>
       </c>
@@ -1908,118 +1910,115 @@
       <c r="P18" s="3"/>
     </row>
     <row r="19" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="78" t="s">
+      <c r="B19" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="69" t="s">
+      <c r="C19" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="D19" s="79" t="s">
+      <c r="D19" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="E19" s="68"/>
-      <c r="F19" s="70"/>
-      <c r="H19" s="73" t="s">
+      <c r="E19" s="56"/>
+      <c r="F19" s="58"/>
+      <c r="H19" s="59" t="s">
         <v>54</v>
       </c>
       <c r="I19" s="53"/>
-      <c r="J19" s="74" t="s">
+      <c r="J19" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="K19" s="75" t="s">
+      <c r="K19" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="L19" s="74" t="s">
+      <c r="L19" s="60" t="s">
         <v>43</v>
       </c>
       <c r="M19" s="53"/>
       <c r="N19" s="54"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B20" s="76">
+      <c r="B20" s="62">
         <v>100</v>
       </c>
-      <c r="C20" s="80">
+      <c r="C20" s="66">
         <f>(24*32/4)</f>
         <v>192</v>
       </c>
-      <c r="D20" s="68" t="s">
+      <c r="D20" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="68"/>
-      <c r="F20" s="70"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="58"/>
       <c r="H20" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="I20" s="71"/>
-      <c r="J20" s="72" t="s">
+      <c r="I20" s="17"/>
+      <c r="J20" t="s">
         <v>44</v>
       </c>
-      <c r="K20" s="65">
+      <c r="K20" s="30">
         <v>30</v>
       </c>
-      <c r="L20" s="72" t="s">
+      <c r="L20" t="s">
         <v>46</v>
       </c>
-      <c r="M20" s="72"/>
       <c r="N20" s="48"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B21" s="83" t="str">
-        <f t="shared" ref="B21:B49" si="17">DEC2HEX(HEX2DEC(B20)+C20)</f>
+      <c r="B21" s="67" t="str">
+        <f t="shared" ref="B21:B47" si="17">DEC2HEX(HEX2DEC(B20)+C20)</f>
         <v>1C0</v>
       </c>
       <c r="C21" s="33">
         <v>64</v>
       </c>
-      <c r="D21" s="84" t="s">
+      <c r="D21" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="E21" s="85"/>
-      <c r="F21" s="86"/>
+      <c r="E21" s="69"/>
+      <c r="F21" s="70"/>
       <c r="H21" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="71"/>
-      <c r="J21" s="72" t="s">
+      <c r="I21" s="17"/>
+      <c r="J21" t="s">
         <v>45</v>
       </c>
-      <c r="K21" s="65">
+      <c r="K21" s="30">
         <v>64</v>
       </c>
-      <c r="L21" s="72" t="s">
+      <c r="L21" t="s">
         <v>46</v>
       </c>
-      <c r="M21" s="72"/>
       <c r="N21" s="48"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B22" s="83" t="str">
+      <c r="B22" s="75" t="str">
         <f t="shared" si="17"/>
         <v>200</v>
       </c>
-      <c r="C22" s="33">
+      <c r="C22" s="76">
         <v>256</v>
       </c>
-      <c r="D22" s="85" t="s">
+      <c r="D22" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="85"/>
-      <c r="F22" s="86"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="78"/>
       <c r="H22" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="I22" s="71"/>
-      <c r="J22" s="72" t="s">
+      <c r="I22" s="17"/>
+      <c r="J22" t="s">
         <v>48</v>
       </c>
-      <c r="K22" s="65">
+      <c r="K22" s="30">
         <v>64</v>
       </c>
-      <c r="L22" s="72" t="s">
+      <c r="L22" t="s">
         <v>47</v>
       </c>
-      <c r="M22" s="72"/>
       <c r="N22" s="48"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.35">
@@ -2027,28 +2026,26 @@
         <f t="shared" si="17"/>
         <v>300</v>
       </c>
-      <c r="C23" s="65">
+      <c r="C23" s="30">
         <v>192</v>
       </c>
-      <c r="D23" s="72" t="s">
+      <c r="D23" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="72"/>
       <c r="F23" s="48"/>
       <c r="H23" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="I23" s="71"/>
-      <c r="J23" s="72" t="s">
+      <c r="I23" s="17"/>
+      <c r="J23" t="s">
         <v>50</v>
       </c>
-      <c r="K23" s="65">
+      <c r="K23" s="30">
         <v>44</v>
       </c>
-      <c r="L23" s="72" t="s">
+      <c r="L23" t="s">
         <v>52</v>
       </c>
-      <c r="M23" s="72"/>
       <c r="N23" s="48"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.35">
@@ -2056,44 +2053,42 @@
         <f t="shared" si="17"/>
         <v>3C0</v>
       </c>
-      <c r="C24" s="65">
+      <c r="C24" s="30">
         <f>$D$8</f>
         <v>32</v>
       </c>
-      <c r="D24" s="77" t="s">
+      <c r="D24" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="E24" s="72"/>
       <c r="F24" s="48"/>
       <c r="H24" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="I24" s="71"/>
-      <c r="J24" s="72" t="s">
+      <c r="I24" s="17"/>
+      <c r="J24" t="s">
         <v>51</v>
       </c>
-      <c r="K24" s="65">
+      <c r="K24" s="30">
         <v>12</v>
       </c>
-      <c r="L24" s="72" t="s">
+      <c r="L24" t="s">
         <v>53</v>
       </c>
-      <c r="M24" s="72"/>
       <c r="N24" s="48"/>
     </row>
     <row r="25" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="83" t="str">
+      <c r="B25" s="67" t="str">
         <f t="shared" si="17"/>
         <v>3E0</v>
       </c>
       <c r="C25" s="33">
         <v>32</v>
       </c>
-      <c r="D25" s="85" t="s">
+      <c r="D25" s="69" t="s">
         <v>71</v>
       </c>
-      <c r="E25" s="85"/>
-      <c r="F25" s="86"/>
+      <c r="E25" s="69"/>
+      <c r="F25" s="70"/>
       <c r="H25" s="49" t="s">
         <v>67</v>
       </c>
@@ -2101,7 +2096,7 @@
       <c r="J25" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="K25" s="92">
+      <c r="K25" s="16">
         <v>20</v>
       </c>
       <c r="L25" s="51" t="s">
@@ -2115,32 +2110,28 @@
         <f t="shared" si="17"/>
         <v>400</v>
       </c>
-      <c r="C26" s="65">
+      <c r="C26" s="30">
         <v>480</v>
       </c>
-      <c r="D26" s="72" t="s">
+      <c r="D26" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="72"/>
       <c r="F26" s="48"/>
-      <c r="H26" s="71"/>
-      <c r="I26" s="71"/>
-      <c r="J26" s="72"/>
-      <c r="K26" s="65"/>
-      <c r="L26" s="72"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="K26" s="30"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B27" s="47" t="str">
         <f t="shared" si="17"/>
         <v>5E0</v>
       </c>
-      <c r="C27" s="65">
+      <c r="C27" s="30">
         <v>48</v>
       </c>
-      <c r="D27" s="72" t="s">
+      <c r="D27" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="72"/>
       <c r="F27" s="48"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.35">
@@ -2148,85 +2139,83 @@
         <f t="shared" si="17"/>
         <v>610</v>
       </c>
-      <c r="C28" s="65">
+      <c r="C28" s="30">
         <v>384</v>
       </c>
-      <c r="D28" s="72" t="s">
+      <c r="D28" t="s">
         <v>20</v>
       </c>
-      <c r="E28" s="72"/>
       <c r="F28" s="48"/>
+      <c r="I28" s="55"/>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="47" t="str">
         <f t="shared" si="17"/>
         <v>790</v>
       </c>
-      <c r="C29" s="65">
+      <c r="C29" s="30">
         <v>96</v>
       </c>
-      <c r="D29" s="72" t="s">
+      <c r="D29" t="s">
         <v>58</v>
       </c>
-      <c r="E29" s="72"/>
       <c r="F29" s="48"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B30" s="83" t="str">
+      <c r="B30" s="67" t="str">
         <f t="shared" si="17"/>
         <v>7F0</v>
       </c>
       <c r="C30" s="33">
         <v>16</v>
       </c>
-      <c r="D30" s="84" t="s">
+      <c r="D30" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="E30" s="85"/>
-      <c r="F30" s="86"/>
+      <c r="E30" s="69"/>
+      <c r="F30" s="70"/>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B31" s="47" t="str">
+      <c r="B31" s="79" t="str">
         <f t="shared" si="17"/>
         <v>800</v>
       </c>
-      <c r="C31" s="65">
+      <c r="C31" s="80">
         <v>128</v>
       </c>
-      <c r="D31" s="72" t="s">
+      <c r="D31" s="81" t="s">
         <v>29</v>
       </c>
-      <c r="E31" s="72"/>
-      <c r="F31" s="48"/>
+      <c r="E31" s="81"/>
+      <c r="F31" s="82"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B32" s="47" t="str">
         <f t="shared" si="17"/>
         <v>880</v>
       </c>
-      <c r="C32" s="65">
+      <c r="C32" s="30">
         <v>64</v>
       </c>
-      <c r="D32" s="77" t="s">
+      <c r="D32" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="E32" s="72"/>
       <c r="F32" s="48"/>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B33" s="83" t="str">
+      <c r="B33" s="75" t="str">
         <f t="shared" si="17"/>
         <v>8C0</v>
       </c>
-      <c r="C33" s="33">
+      <c r="C33" s="76">
         <f>2*$D$8</f>
         <v>64</v>
       </c>
-      <c r="D33" s="85" t="s">
+      <c r="D33" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="E33" s="85"/>
-      <c r="F33" s="86"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="78"/>
       <c r="H33" s="55"/>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.35">
@@ -2234,28 +2223,27 @@
         <f t="shared" si="17"/>
         <v>900</v>
       </c>
-      <c r="C34" s="65">
+      <c r="C34" s="30">
         <v>960</v>
       </c>
-      <c r="D34" s="72" t="s">
+      <c r="D34" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="72"/>
       <c r="F34" s="48"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B35" s="83" t="str">
+      <c r="B35" s="67" t="str">
         <f t="shared" si="17"/>
         <v>CC0</v>
       </c>
       <c r="C35" s="33">
         <v>64</v>
       </c>
-      <c r="D35" s="85" t="s">
+      <c r="D35" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="85"/>
-      <c r="F35" s="86"/>
+      <c r="E35" s="69"/>
+      <c r="F35" s="70"/>
       <c r="H35" s="55"/>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.35">
@@ -2263,13 +2251,12 @@
         <f t="shared" si="17"/>
         <v>D00</v>
       </c>
-      <c r="C36" s="65">
+      <c r="C36" s="30">
         <v>32</v>
       </c>
-      <c r="D36" s="77" t="s">
+      <c r="D36" s="63" t="s">
         <v>70</v>
       </c>
-      <c r="E36" s="72"/>
       <c r="F36" s="48"/>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.35">
@@ -2277,28 +2264,27 @@
         <f t="shared" si="17"/>
         <v>D20</v>
       </c>
-      <c r="C37" s="81">
+      <c r="C37" s="30">
         <v>64</v>
       </c>
-      <c r="D37" s="82" t="s">
+      <c r="D37" t="s">
         <v>60</v>
       </c>
-      <c r="E37" s="72"/>
       <c r="F37" s="48"/>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B38" s="83" t="str">
+      <c r="B38" s="75" t="str">
         <f t="shared" si="17"/>
         <v>D60</v>
       </c>
-      <c r="C38" s="87">
+      <c r="C38" s="76">
         <v>160</v>
       </c>
-      <c r="D38" s="88" t="s">
+      <c r="D38" s="77" t="s">
         <v>61</v>
       </c>
-      <c r="E38" s="85"/>
-      <c r="F38" s="86"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="78"/>
       <c r="H38" s="3"/>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.35">
@@ -2306,13 +2292,12 @@
         <f t="shared" si="17"/>
         <v>E00</v>
       </c>
-      <c r="C39" s="65">
+      <c r="C39" s="30">
         <v>384</v>
       </c>
-      <c r="D39" s="77" t="s">
+      <c r="D39" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="E39" s="72"/>
       <c r="F39" s="48"/>
       <c r="H39" s="3"/>
     </row>
@@ -2321,55 +2306,53 @@
         <f t="shared" si="17"/>
         <v>F80</v>
       </c>
-      <c r="C40" s="65">
+      <c r="C40" s="30">
         <v>32</v>
       </c>
-      <c r="D40" s="77" t="s">
+      <c r="D40" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="E40" s="72"/>
       <c r="F40" s="48"/>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B41" s="83" t="str">
+      <c r="B41" s="67" t="str">
         <f t="shared" si="17"/>
         <v>FA0</v>
       </c>
       <c r="C41" s="33">
         <v>96</v>
       </c>
-      <c r="D41" s="84" t="s">
+      <c r="D41" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="E41" s="85"/>
-      <c r="F41" s="86"/>
+      <c r="E41" s="69"/>
+      <c r="F41" s="70"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B42" s="47" t="str">
+      <c r="B42" s="79" t="str">
         <f t="shared" si="17"/>
         <v>1000</v>
       </c>
-      <c r="C42" s="65">
+      <c r="C42" s="80">
         <v>144</v>
       </c>
-      <c r="D42" s="77" t="s">
+      <c r="D42" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="E42" s="72"/>
-      <c r="F42" s="48"/>
+      <c r="E42" s="81"/>
+      <c r="F42" s="82"/>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B43" s="47" t="str">
         <f t="shared" si="17"/>
         <v>1090</v>
       </c>
-      <c r="C43" s="65">
+      <c r="C43" s="30">
         <v>48</v>
       </c>
-      <c r="D43" s="77" t="s">
+      <c r="D43" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="E43" s="72"/>
       <c r="F43" s="48"/>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.35">
@@ -2377,13 +2360,12 @@
         <f t="shared" si="17"/>
         <v>10C0</v>
       </c>
-      <c r="C44" s="65">
+      <c r="C44" s="30">
         <v>32</v>
       </c>
-      <c r="D44" s="77" t="s">
+      <c r="D44" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="E44" s="72"/>
       <c r="F44" s="48"/>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.35">
@@ -2391,56 +2373,54 @@
         <f t="shared" si="17"/>
         <v>10E0</v>
       </c>
-      <c r="C45" s="65">
+      <c r="C45" s="30">
         <v>12</v>
       </c>
-      <c r="D45" s="77" t="s">
+      <c r="D45" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="E45" s="72"/>
       <c r="F45" s="48"/>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B46" s="83" t="str">
+      <c r="B46" s="67" t="str">
         <f t="shared" si="17"/>
         <v>10EC</v>
       </c>
       <c r="C46" s="33">
         <v>20</v>
       </c>
-      <c r="D46" s="84" t="s">
+      <c r="D46" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="E46" s="85"/>
-      <c r="F46" s="86"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="70"/>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B47" s="47" t="str">
         <f t="shared" si="17"/>
         <v>1100</v>
       </c>
-      <c r="C47" s="89">
+      <c r="C47" s="71">
         <f>HEX2DEC(B49)-HEX2DEC(B47)</f>
         <v>7680</v>
       </c>
-      <c r="D47" s="90" t="s">
+      <c r="D47" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="E47" s="90"/>
-      <c r="F47" s="91"/>
+      <c r="E47" s="72"/>
+      <c r="F47" s="73"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.35">
-      <c r="B48" s="93" t="str">
+      <c r="B48" s="74" t="str">
         <f t="shared" ref="B48" si="18">DEC2HEX(HEX2DEC(B49)-C48)</f>
         <v>2BA0</v>
       </c>
-      <c r="C48" s="65">
+      <c r="C48" s="30">
         <v>864</v>
       </c>
-      <c r="D48" s="72" t="s">
+      <c r="D48" t="s">
         <v>64</v>
       </c>
-      <c r="E48" s="72"/>
       <c r="F48" s="48"/>
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.35">
@@ -2448,17 +2428,16 @@
         <f t="shared" ref="B49:B51" si="19">DEC2HEX(HEX2DEC(B50)-C49)</f>
         <v>2F00</v>
       </c>
-      <c r="C49" s="65">
+      <c r="C49" s="30">
         <v>96</v>
       </c>
-      <c r="D49" s="72" t="s">
+      <c r="D49" t="s">
         <v>66</v>
       </c>
-      <c r="E49" s="72"/>
       <c r="F49" s="48"/>
     </row>
     <row r="50" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B50" s="83" t="str">
+      <c r="B50" s="67" t="str">
         <f>DEC2HEX(HEX2DEC(B51)-C50)</f>
         <v>2F60</v>
       </c>
@@ -2466,25 +2445,24 @@
         <f>$D$11</f>
         <v>224</v>
       </c>
-      <c r="D50" s="85" t="s">
+      <c r="D50" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="E50" s="85"/>
-      <c r="F50" s="86"/>
+      <c r="E50" s="69"/>
+      <c r="F50" s="70"/>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B51" s="47" t="str">
         <f t="shared" si="19"/>
         <v>3040</v>
       </c>
-      <c r="C51" s="65">
+      <c r="C51" s="30">
         <f>64*31</f>
         <v>1984</v>
       </c>
-      <c r="D51" s="71" t="s">
+      <c r="D51" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="E51" s="72"/>
       <c r="F51" s="48"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.35">
@@ -2492,14 +2470,13 @@
         <f t="shared" ref="B52" si="20">DEC2HEX(HEX2DEC(B53)-C52)</f>
         <v>3800</v>
       </c>
-      <c r="C52" s="65">
+      <c r="C52" s="30">
         <f>2048</f>
         <v>2048</v>
       </c>
-      <c r="D52" s="71" t="s">
+      <c r="D52" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="E52" s="72"/>
       <c r="F52" s="48"/>
     </row>
     <row r="53" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">

</xml_diff>